<commit_message>
Actualizacion estado de cu
</commit_message>
<xml_diff>
--- a/Documentación/RESUMEN Estado de CU.xlsx
+++ b/Documentación/RESUMEN Estado de CU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/74d3b8e2b788a22f/Escritorio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Desktop\VitalSY-main\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="563" documentId="11_F25DC773A252ABDACC1048D4E15D6CC05BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5916211F-9F9A-4F5C-B665-59E7B0FC23F0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87ABDF90-B28B-4042-A1DB-0CD141D31FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN 1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="122">
   <si>
     <t>Proyecto: VitalSY</t>
   </si>
@@ -249,27 +249,6 @@
     <t>Se hacen ajustes vizuales.</t>
   </si>
   <si>
-    <t>Se genera un registro de perfil basico pero operable</t>
-  </si>
-  <si>
-    <t>Se genera gestión de perfil completa, pendiente a reajustes en caso de.</t>
-  </si>
-  <si>
-    <t>No se registran mayores cambios desde el ultimo reporte.</t>
-  </si>
-  <si>
-    <t>Se establece un registro simulado con opciónes de reporte especificas a disposición del paciente.</t>
-  </si>
-  <si>
-    <t>No se registran mayores cambios.</t>
-  </si>
-  <si>
-    <t>No se registran cambios mayores.</t>
-  </si>
-  <si>
-    <t>Ho se registran cambios mayores.</t>
-  </si>
-  <si>
     <t>Los datos se tiene con certeza si son fijos o tienden a cambiar con el tiempo.</t>
   </si>
   <si>
@@ -292,6 +271,129 @@
   </si>
   <si>
     <t>Se requiere entrenar a la IA para de sea capaz de dar más respuestas dependiendo de las glicemias.</t>
+  </si>
+  <si>
+    <t>CU 14</t>
+  </si>
+  <si>
+    <t>CU 15</t>
+  </si>
+  <si>
+    <t>CU 16</t>
+  </si>
+  <si>
+    <t>CU 17</t>
+  </si>
+  <si>
+    <t>CU 18</t>
+  </si>
+  <si>
+    <t>CU 19</t>
+  </si>
+  <si>
+    <t>CU 20</t>
+  </si>
+  <si>
+    <t>Recuperación de Contraseña mediante Correo</t>
+  </si>
+  <si>
+    <t>Se implementó el flujo completo de recuperación con envío de correo seguro (Mailtrap/JavaMailSender en backend) y formulario de cambio de contraseña en frontend.</t>
+  </si>
+  <si>
+    <t>Sincronización Automática con LibreLinkUp (Sensor Cloud)</t>
+  </si>
+  <si>
+    <t>Usuario (Paciente) / Sensor de medición / Abbott Cloud</t>
+  </si>
+  <si>
+    <t>Conexión directa mediante scraping/REST a la API de LibreLinkUp (Abbott) con redirección regional y tareas programadas en segundo plano cada 5 minutos.</t>
+  </si>
+  <si>
+    <t>Asistente Virtual / Chat Clínico Interactivo con IA</t>
+  </si>
+  <si>
+    <t>Usuario (Paciente) / Engine de IA (Gemini)</t>
+  </si>
+  <si>
+    <t>Chatbot integrado que permite realizar consultas en lenguaje natural y entrada de voz (Speech-to-Text con Capacitor) analizando el contexto de los últimos 7 días de bitácora del paciente.</t>
+  </si>
+  <si>
+    <t>Análisis Predictivo Causal de Patrones y Alertas con IA</t>
+  </si>
+  <si>
+    <t>Análisis predictivo de 7 días que evalúa causalidad en la bitácora para predecir niveles de riesgo (alto/medio/bajo), alertar riesgos inminentes a 4 horas y recomendar acciones.</t>
+  </si>
+  <si>
+    <t>Panel de Control y Gestión Administrativa de Usuarios</t>
+  </si>
+  <si>
+    <t>Administrador</t>
+  </si>
+  <si>
+    <t>Panel web completo para auditar usuarios, ver estadísticas globales del sistema, activar/suspender cuentas y forzar restablecimiento de contraseñas.</t>
+  </si>
+  <si>
+    <t>Monitoreo Clínico de Pacientes (Gráfico de Glucemia)</t>
+  </si>
+  <si>
+    <t>Vista detallada de pacientes para administradores, incluyendo perfil basal y gráfica interactiva (con ng2-charts) de la evolución histórica de glucemias.</t>
+  </si>
+  <si>
+    <t>Digitalización Multimodal de Pautas Médicas (OCR con IA)</t>
+  </si>
+  <si>
+    <t>Usuario (Paciente) / Engine de IA (Gemini OCR)</t>
+  </si>
+  <si>
+    <t>OCR multimodal mediante Gemini que permite cargar una fotografía de la receta médica e identificar y guardar automáticamente la matriz de escalas de dosis de insulina.</t>
+  </si>
+  <si>
+    <t>Autenticación JWT completamente operativa, endpoints de registro e inicio de sesión y persistencia local del token.</t>
+  </si>
+  <si>
+    <t>Gestión de perfil completa con datos basales (nombre, peso, altura, tipos de insulina) y sincronización con local storage y base de datos.</t>
+  </si>
+  <si>
+    <t>Coeficientes médicos (Ratio IC y Factor de Sensibilidad) implementados en la base de datos y configurables desde la vista de perfil.</t>
+  </si>
+  <si>
+    <t>Sensor de medición</t>
+  </si>
+  <si>
+    <t>Registro de lecturas con fecha, valor, carbohidratos, comentarios y tendencia, sincronizado automáticamente por LibreLinkUp en segundo plano.</t>
+  </si>
+  <si>
+    <t>Permite registrar carbohidratos consumidos, notas del alimento y momento de la ingesta directamente desde el panel de registro de glucosa.</t>
+  </si>
+  <si>
+    <t>Implementada calculadora inteligente con soporte a matrices de insulina fija (pauta médica) y fallback algorítmico tradicional.</t>
+  </si>
+  <si>
+    <t>Integración de análisis clínico reactivo de glucosa mediante Gemini API. La recomendación de IA se guarda adjunta a la lectura.</t>
+  </si>
+  <si>
+    <t>Envío automatizado de alertas críticas (Hiper/Hipoglucemia) y de riesgos altos de IA mediante notificaciones push locales nativas y ventanas de alerta visual.</t>
+  </si>
+  <si>
+    <t>Pantalla de historial completa con agrupación diaria de eventos, orden descendente, estados de rango e interacción táctil (accordions y refresh).</t>
+  </si>
+  <si>
+    <t>Despliegue en dashboard de gráfico lineal interactivo de glucosa y barra tricolor de distribución de Tiempo en Rango (TIR) con cálculo dinámico.</t>
+  </si>
+  <si>
+    <t>Exportación completa de reportes médicos en PDF que incluyen datos del paciente, resumen estadístico de 30 días, listado de lecturas y gráfico AGP.</t>
+  </si>
+  <si>
+    <t>Preferencia de recordatorios de comidas integrada en el perfil y guardada en el backend. Pendiente lógica de alertas temporizadas programadas.</t>
+  </si>
+  <si>
+    <t>Pendiente implementar el servicio scheduler en segundo plano para disparar las alertas temporizadas.</t>
+  </si>
+  <si>
+    <t>Límites configurados en base de datos e integrados en el backend. Los límites se utilizan en el dashboard para calcular el TIR, pero falta agregarlos al formulario del perfil.</t>
+  </si>
+  <si>
+    <t>Falta exponer los campos en la vista de configuración del perfil del usuario para edición manual.</t>
   </si>
 </sst>
 </file>
@@ -387,7 +489,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -432,9 +534,6 @@
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -471,11 +570,8 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -492,10 +588,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -762,7 +854,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B4:I22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
@@ -1170,7 +1262,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66617FB-57B0-4DDD-AABF-48FED053008F}">
   <dimension ref="B1:I20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
@@ -1307,7 +1399,7 @@
         <v>56</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1333,7 +1425,7 @@
         <v>58</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1355,11 +1447,11 @@
       <c r="G12" s="9">
         <v>0.38</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I12" s="24" t="s">
-        <v>82</v>
+      <c r="I12" s="23" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
@@ -1385,7 +1477,7 @@
         <v>60</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1578,7 +1670,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387406B4-0345-48AA-AD46-BF1413BF8B45}">
   <dimension ref="B2:I20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
@@ -1640,51 +1732,51 @@
       </c>
     </row>
     <row r="8" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B8" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C8" s="17" t="s">
+      <c r="B8" s="20">
+        <v>46161</v>
+      </c>
+      <c r="C8" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="22" t="s">
         <v>39</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="17">
         <v>0.6</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="23" t="s">
         <v>65</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="2:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B9" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C9" s="19" t="s">
+      <c r="B9" s="24">
+        <v>46161</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="26" t="s">
         <v>39</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="19">
         <v>0.68</v>
       </c>
-      <c r="H9" s="28" t="s">
+      <c r="H9" s="27" t="s">
         <v>66</v>
       </c>
       <c r="I9" s="14" t="s">
@@ -1692,25 +1784,25 @@
       </c>
     </row>
     <row r="10" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B10" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C10" s="17" t="s">
+      <c r="B10" s="20">
+        <v>46161</v>
+      </c>
+      <c r="C10" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="22" t="s">
         <v>39</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="17">
         <v>0.79</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="23" t="s">
         <v>67</v>
       </c>
       <c r="I10" s="3" t="s">
@@ -1718,77 +1810,77 @@
       </c>
     </row>
     <row r="11" spans="2:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="B11" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C11" s="19" t="s">
+      <c r="B11" s="24">
+        <v>46161</v>
+      </c>
+      <c r="C11" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="E11" s="26" t="s">
         <v>42</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="19">
         <v>0.52</v>
       </c>
-      <c r="H11" s="28" t="s">
+      <c r="H11" s="27" t="s">
         <v>68</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B12" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C12" s="17" t="s">
+      <c r="B12" s="20">
+        <v>46161</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="22" t="s">
         <v>39</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="17">
         <v>0.54</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="23" t="s">
         <v>69</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B13" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C13" s="19" t="s">
+      <c r="B13" s="24">
+        <v>46161</v>
+      </c>
+      <c r="C13" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="26" t="s">
         <v>39</v>
       </c>
       <c r="F13" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="19">
         <v>0.23</v>
       </c>
-      <c r="H13" s="28" t="s">
+      <c r="H13" s="27" t="s">
         <v>70</v>
       </c>
       <c r="I13" s="14" t="s">
@@ -1796,51 +1888,51 @@
       </c>
     </row>
     <row r="14" spans="2:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="B14" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C14" s="17" t="s">
+      <c r="B14" s="20">
+        <v>46161</v>
+      </c>
+      <c r="C14" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="E14" s="22" t="s">
         <v>41</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="17">
         <v>0.4</v>
       </c>
-      <c r="H14" s="24" t="s">
+      <c r="H14" s="23" t="s">
         <v>71</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B15" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C15" s="19" t="s">
+      <c r="B15" s="24">
+        <v>46161</v>
+      </c>
+      <c r="C15" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="E15" s="26" t="s">
         <v>40</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="19">
         <v>0</v>
       </c>
-      <c r="H15" s="28" t="s">
+      <c r="H15" s="27" t="s">
         <v>70</v>
       </c>
       <c r="I15" s="14" t="s">
@@ -1848,25 +1940,25 @@
       </c>
     </row>
     <row r="16" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C16" s="17" t="s">
+      <c r="B16" s="20">
+        <v>46161</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="22" t="s">
         <v>39</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="17">
         <v>0.67</v>
       </c>
-      <c r="H16" s="24" t="s">
+      <c r="H16" s="23" t="s">
         <v>72</v>
       </c>
       <c r="I16" s="3" t="s">
@@ -1874,25 +1966,25 @@
       </c>
     </row>
     <row r="17" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B17" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C17" s="19" t="s">
+      <c r="B17" s="24">
+        <v>46161</v>
+      </c>
+      <c r="C17" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="26" t="s">
         <v>39</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="19">
         <v>0</v>
       </c>
-      <c r="H17" s="28" t="s">
+      <c r="H17" s="27" t="s">
         <v>70</v>
       </c>
       <c r="I17" s="14" t="s">
@@ -1900,25 +1992,25 @@
       </c>
     </row>
     <row r="18" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B18" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C18" s="17" t="s">
+      <c r="B18" s="20">
+        <v>46161</v>
+      </c>
+      <c r="C18" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="22" t="s">
         <v>39</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="17">
         <v>0.1</v>
       </c>
-      <c r="H18" s="24" t="s">
+      <c r="H18" s="23" t="s">
         <v>70</v>
       </c>
       <c r="I18" s="3" t="s">
@@ -1926,25 +2018,25 @@
       </c>
     </row>
     <row r="19" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C19" s="19" t="s">
+      <c r="B19" s="24">
+        <v>46161</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="26" t="s">
         <v>39</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G19" s="20">
+      <c r="G19" s="19">
         <v>0</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="H19" s="27" t="s">
         <v>70</v>
       </c>
       <c r="I19" s="14" t="s">
@@ -1952,25 +2044,25 @@
       </c>
     </row>
     <row r="20" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B20" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C20" s="17" t="s">
+      <c r="B20" s="20">
+        <v>46161</v>
+      </c>
+      <c r="C20" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="22" t="s">
         <v>39</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="17">
         <v>0</v>
       </c>
-      <c r="H20" s="24" t="s">
+      <c r="H20" s="23" t="s">
         <v>70</v>
       </c>
       <c r="I20" s="3" t="s">
@@ -1984,17 +2076,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90B11430-C3BA-45D5-9916-571D2BDFBBC3}">
-  <dimension ref="B2:I20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:I28"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="43.42578125" customWidth="1"/>
-    <col min="5" max="5" width="29.5703125" customWidth="1"/>
+    <col min="4" max="4" width="40.5703125" customWidth="1"/>
+    <col min="5" max="5" width="44.7109375" customWidth="1"/>
     <col min="6" max="6" width="26.7109375" customWidth="1"/>
-    <col min="7" max="7" width="24.7109375" customWidth="1"/>
-    <col min="8" max="8" width="19.7109375" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="41.28515625" customWidth="1"/>
+    <col min="9" max="9" width="23.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
@@ -2046,343 +2138,528 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B8" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C8" s="17" t="s">
+    <row r="8" spans="2:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="B8" s="5">
+        <v>46161</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="8" t="s">
         <v>39</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="9">
         <v>1</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I8" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="9" spans="2:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B9" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C9" s="19" t="s">
+      <c r="B9" s="10">
+        <v>46161</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="13" t="s">
         <v>39</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="15">
         <v>1</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="I9" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="I9" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="10" spans="2:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B10" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C10" s="17" t="s">
+      <c r="B10" s="5">
+        <v>46161</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="8" t="s">
         <v>39</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="9">
         <v>1</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I10" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="B11" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C11" s="19" t="s">
+      <c r="B11" s="10">
+        <v>46161</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="27" t="s">
-        <v>42</v>
+      <c r="E11" s="13" t="s">
+        <v>109</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="20">
-        <v>0.6</v>
+      <c r="G11" s="15">
+        <v>1</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="I11" s="29" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="B12" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C12" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B12" s="5">
+        <v>46161</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="8" t="s">
         <v>39</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="9">
         <v>1</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="I12" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B13" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C13" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="B13" s="10">
+        <v>46161</v>
+      </c>
+      <c r="C13" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="13" t="s">
         <v>39</v>
       </c>
       <c r="F13" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G13" s="20">
-        <v>0.23</v>
+      <c r="G13" s="15">
+        <v>1</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="I13" s="29" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B14" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C14" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B14" s="5">
+        <v>46161</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="E14" s="8" t="s">
         <v>41</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G14" s="18">
-        <v>0.46</v>
+      <c r="G14" s="9">
+        <v>1</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I14" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B15" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C15" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B15" s="10">
+        <v>46161</v>
+      </c>
+      <c r="C15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="E15" s="13" t="s">
         <v>40</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="G15" s="20">
-        <v>0</v>
+      <c r="G15" s="15">
+        <v>1</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="I15" s="29" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C16" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B16" s="5">
+        <v>46161</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="8" t="s">
         <v>39</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G16" s="18">
-        <v>0.7</v>
+      <c r="G16" s="9">
+        <v>1</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="I16" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B17" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C17" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B17" s="10">
+        <v>46161</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="13" t="s">
         <v>39</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="G17" s="20">
-        <v>0</v>
+      <c r="G17" s="15">
+        <v>1</v>
       </c>
       <c r="H17" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="I17" s="29" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B18" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C18" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B18" s="5">
+        <v>46161</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="8" t="s">
         <v>39</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G18" s="18">
-        <v>0.1</v>
-      </c>
-      <c r="H18" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="I18" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19" s="25">
-        <v>46161</v>
-      </c>
-      <c r="C19" s="19" t="s">
+      <c r="G18" s="9">
+        <v>1</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="B19" s="10">
+        <v>46161</v>
+      </c>
+      <c r="C19" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="13" t="s">
         <v>39</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G19" s="20">
-        <v>0</v>
+      <c r="G19" s="15">
+        <v>0.15</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="I19" s="29" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B20" s="21">
-        <v>46161</v>
-      </c>
-      <c r="C20" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="5">
+        <v>46188</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="8" t="s">
         <v>39</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G20" s="18">
-        <v>0</v>
-      </c>
-      <c r="H20" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="I20" s="16" t="s">
-        <v>54</v>
-      </c>
+      <c r="G20" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="10">
+        <v>46188</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="G21" s="15">
+        <v>1</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="5">
+        <v>46188</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G22" s="9">
+        <v>1</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="10">
+        <v>46188</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="G23" s="15">
+        <v>1</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" ht="84" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="5">
+        <v>46188</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G24" s="9">
+        <v>1</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="10">
+        <v>46188</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="G25" s="15">
+        <v>1</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="5">
+        <v>46188</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G26" s="9">
+        <v>1</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="10">
+        <v>46188</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="G27" s="15">
+        <v>1</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D28" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se actualizan los docuemntos Resumen Estado de CU y Plan de Pruebas a su version final.
</commit_message>
<xml_diff>
--- a/Documentación/RESUMEN Estado de CU.xlsx
+++ b/Documentación/RESUMEN Estado de CU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Desktop\VitalSY-main\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87ABDF90-B28B-4042-A1DB-0CD141D31FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0B77CD-7D25-499A-BF6D-C9DB03CEFF15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="120">
   <si>
     <t>Proyecto: VitalSY</t>
   </si>
@@ -384,16 +384,10 @@
     <t>Exportación completa de reportes médicos en PDF que incluyen datos del paciente, resumen estadístico de 30 días, listado de lecturas y gráfico AGP.</t>
   </si>
   <si>
-    <t>Preferencia de recordatorios de comidas integrada en el perfil y guardada en el backend. Pendiente lógica de alertas temporizadas programadas.</t>
-  </si>
-  <si>
-    <t>Pendiente implementar el servicio scheduler en segundo plano para disparar las alertas temporizadas.</t>
-  </si>
-  <si>
     <t>Límites configurados en base de datos e integrados en el backend. Los límites se utilizan en el dashboard para calcular el TIR, pero falta agregarlos al formulario del perfil.</t>
   </si>
   <si>
-    <t>Falta exponer los campos en la vista de configuración del perfil del usuario para edición manual.</t>
+    <t>Preferencia de recordatorios de comidas integrada en el perfil y guardada en el backend. Lógica de alertas temporizadas programadas.</t>
   </si>
 </sst>
 </file>
@@ -2424,7 +2418,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="2:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B19" s="10">
         <v>46161</v>
       </c>
@@ -2441,13 +2435,13 @@
         <v>4</v>
       </c>
       <c r="G19" s="15">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>119</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2467,13 +2461,13 @@
         <v>2</v>
       </c>
       <c r="G20" s="9">
-        <v>0.05</v>
+        <v>1</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>121</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="96" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>